<commit_message>
Update NREL-118 data, refining translation from original data source
Update InOutModule to newest version
Add xlrd to environment (for reading Excels directly)
</commit_message>
<xml_diff>
--- a/data/NREL-118/Data_Sources.xlsx
+++ b/data/NREL-118/Data_Sources.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5703125" customWidth="1" min="1" max="1"/>
@@ -969,7 +969,205 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Adjusted MaxProd multiplied by DisEffic (since it is not present any more</t>
+          <t>Adjusted MaxProd multiplied by DisEffic (since it is not present any more)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>hydro-hourly-inflows</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/input-files/Hydro/Hydro [XX].csv</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>45979</v>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Inflow data from individual, hourly entries in NREL-118 data set</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>hydro-monthly-fixed-inflows</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/additional-files-mti-118/Hydro_nondipatchable.csv</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>45979</v>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Inflow data from monthly fixed (non-dispatchable) entries in NREL-118 data set</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>plexos-monthly-budgets</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/plexos-export.xls</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>45979</v>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>Inflow data from plexos-export, where a 'monthly budget' is added to the hydro reservoir at the first hour of each month</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>vres-generators</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/additional-files-mti-118/Generators.csv</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>45980</v>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Max capacity and node information from generators.csv, OMVarCost and FirmCapCoef chosen arbitrarily. Note that those Hydro generators with monthly budgets are found in Power_Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>hydro-generators-monthly-budget</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/additional-files-mti-118/Generators.csv</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>45980</v>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Hydro generators with monthly budget that can be dispatched. Max capacity and node information from generators.csv, all other parameters chosen arbitrarily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="10" t="n">
+        <v/>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>vres-profiles</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>NREL-118/input-files/RT/[Solar|Wind]/[Solar|Wind] [XX]RT.csv</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Felix Auer</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>45980</v>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>Capacity factors from NREL-118 Real-Time (RT) data, clipped to be &lt;=100% (some entries would otherwise be up to 130%)</t>
         </is>
       </c>
     </row>

</xml_diff>